<commit_message>
checking in recent changes
</commit_message>
<xml_diff>
--- a/experiment_output/OneCombinedGame/ElapsedTimePerFilesOnebyOneOneCombinedGameFinal.xlsx
+++ b/experiment_output/OneCombinedGame/ElapsedTimePerFilesOnebyOneOneCombinedGameFinal.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\90948045\OneDrive - Western Sydney University\Documents\ThesisTimingData\OneCombinedGame\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://westernsydneyedu-my.sharepoint.com/personal/90948045_westernsydney_edu_au/Documents/Documents/Thesis/OneCombinedGame/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E70BF106-5E46-4C2F-BB40-9F2856F0A843}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="35" documentId="13_ncr:1_{E70BF106-5E46-4C2F-BB40-9F2856F0A843}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B01C7E30-221C-4937-8D9A-365F613A149C}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="11964" xr2:uid="{DD70F422-05DF-4428-95ED-77B35152BC41}"/>
   </bookViews>
@@ -70,9 +70,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="0.000"/>
-  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -104,7 +101,7 @@
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -512,7 +509,7 @@
                       </c:ext>
                     </c:extLst>
                     <c:numCache>
-                      <c:formatCode>0.000</c:formatCode>
+                      <c:formatCode>General</c:formatCode>
                       <c:ptCount val="21"/>
                       <c:pt idx="0">
                         <c:v>0.42379900068044601</c:v>
@@ -1100,7 +1097,7 @@
             <c:numRef>
               <c:f>[1]Windows!$H$2:$H$22</c:f>
               <c:numCache>
-                <c:formatCode>0.000</c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="21"/>
                 <c:pt idx="0">
                   <c:v>0.42379900068044601</c:v>
@@ -1586,7 +1583,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="0.000" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -2114,7 +2111,7 @@
                       </c:ext>
                     </c:extLst>
                     <c:numCache>
-                      <c:formatCode>0.000</c:formatCode>
+                      <c:formatCode>General</c:formatCode>
                       <c:ptCount val="21"/>
                       <c:pt idx="0">
                         <c:v>9.4554035000328399E-2</c:v>
@@ -2715,7 +2712,7 @@
             <c:numRef>
               <c:f>Linux!$H$2:$H$22</c:f>
               <c:numCache>
-                <c:formatCode>0.000</c:formatCode>
+                <c:formatCode>General</c:formatCode>
                 <c:ptCount val="21"/>
                 <c:pt idx="0">
                   <c:v>9.4554035000328399E-2</c:v>
@@ -3200,7 +3197,7 @@
             </a:p>
           </c:txPr>
         </c:title>
-        <c:numFmt formatCode="0.000" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -5633,16 +5630,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>8</xdr:col>
-      <xdr:colOff>30480</xdr:colOff>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>22860</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>83820</xdr:rowOff>
+      <xdr:rowOff>160020</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>18</xdr:col>
-      <xdr:colOff>579120</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>167640</xdr:rowOff>
+      <xdr:col>20</xdr:col>
+      <xdr:colOff>571500</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -6277,6 +6274,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00D03EA6-76E3-4B2E-8D81-518836C45664}">
   <dimension ref="A1:H22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="8" max="8" width="9.109375" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
@@ -6352,7 +6352,7 @@
         <v>2</v>
       </c>
       <c r="G3">
-        <f t="shared" ref="G3:G22" si="0">AVERAGE(A3:E3)</f>
+        <f t="shared" ref="G3:I22" si="0">AVERAGE(A3:E3)</f>
         <v>0.43357236050069281</v>
       </c>
       <c r="H3" s="1">
@@ -6903,8 +6903,12 @@
   <dimension ref="A1:H22"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="5" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.33203125" customWidth="1"/>
+    <col min="2" max="2" width="9.44140625" customWidth="1"/>
+    <col min="3" max="4" width="9.109375" customWidth="1"/>
+    <col min="5" max="5" width="9.5546875" customWidth="1"/>
     <col min="6" max="6" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
@@ -6953,7 +6957,7 @@
         <v>1</v>
       </c>
       <c r="G2">
-        <f t="shared" ref="G2:G22" si="0">AVERAGE(A2:E2)</f>
+        <f t="shared" ref="G2:I22" si="0">AVERAGE(A2:E2)</f>
         <v>9.493907140004007E-2</v>
       </c>
       <c r="H2" s="1">

</xml_diff>